<commit_message>
committed @ 2026-02-19-042910+0000 by tychen@ubuntu
</commit_message>
<xml_diff>
--- a/chapters/04-pandas/Excel_Sample.xlsx
+++ b/chapters/04-pandas/Excel_Sample.xlsx
@@ -425,31 +425,101 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:T5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0.14</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.13</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.12</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.11</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.10</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.9</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.8</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.7</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.6</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.5</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.4</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.3</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.2</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.1</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
@@ -466,12 +536,54 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S2" t="n">
+        <v>2</v>
+      </c>
+      <c r="T2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -483,15 +595,57 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="n">
         <v>4</v>
       </c>
-      <c r="D3" t="n">
+      <c r="R3" t="n">
         <v>5</v>
       </c>
-      <c r="E3" t="n">
+      <c r="S3" t="n">
         <v>6</v>
       </c>
-      <c r="F3" t="n">
+      <c r="T3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -503,15 +657,57 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q4" t="n">
         <v>8</v>
       </c>
-      <c r="D4" t="n">
+      <c r="R4" t="n">
         <v>9</v>
       </c>
-      <c r="E4" t="n">
+      <c r="S4" t="n">
         <v>10</v>
       </c>
-      <c r="F4" t="n">
+      <c r="T4" t="n">
         <v>11</v>
       </c>
     </row>
@@ -523,15 +719,57 @@
         <v>3</v>
       </c>
       <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" t="n">
+        <v>3</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>3</v>
+      </c>
+      <c r="M5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P5" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q5" t="n">
         <v>12</v>
       </c>
-      <c r="D5" t="n">
+      <c r="R5" t="n">
         <v>13</v>
       </c>
-      <c r="E5" t="n">
+      <c r="S5" t="n">
         <v>14</v>
       </c>
-      <c r="F5" t="n">
+      <c r="T5" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
committed @ 2026-05-14-093005-0500 by tcn85@rtsjpl774kw20.managed.mst.edu
</commit_message>
<xml_diff>
--- a/chapters/04-pandas/Excel_Sample.xlsx
+++ b/chapters/04-pandas/Excel_Sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,104 +417,104 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Unnamed: 0.14</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Unnamed: 0.13</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Unnamed: 0.12</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Unnamed: 0.11</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Unnamed: 0.10</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Unnamed: 0.9</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Unnamed: 0.8</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Unnamed: 0.7</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Unnamed: 0.6</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Unnamed: 0.5</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Unnamed: 0.4</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Unnamed: 0.3</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Unnamed: 0.2</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Unnamed: 0.1</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
@@ -588,7 +576,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="n">
@@ -650,7 +638,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="n">
@@ -712,7 +700,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="n">

</xml_diff>

<commit_message>
committed @ 2026-05-17-112720-0500 by tcn85@rtsjpl774kw20.managed.mst.edu
</commit_message>
<xml_diff>
--- a/chapters/04-pandas/Excel_Sample.xlsx
+++ b/chapters/04-pandas/Excel_Sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,104 +429,104 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.14</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.13</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.12</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.11</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.10</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.9</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.8</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.7</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.6</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.5</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.4</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.3</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.2</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.1</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
@@ -576,7 +588,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="n">
@@ -638,7 +650,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="n">
@@ -700,7 +712,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="n">

</xml_diff>